<commit_message>
fix(materiales): correct 51107 thrust bearing count and complete bearing specs
</commit_message>
<xml_diff>
--- a/lista_materiales_scara_sin_3d_sin_fuente_madera_abrazaderas.xlsx
+++ b/lista_materiales_scara_sin_3d_sin_fuente_madera_abrazaderas.xlsx
@@ -549,10 +549,14 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>El tercero puede ser más corto</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
+          <t>J1, J2, J3 y Z</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>El de J3 puede ser el corto de 24 mm</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -584,7 +588,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Arduino Uno</t>
+          <t>Arduino Mega 2560</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -592,11 +596,15 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>R3 o equivalente</t>
+          <t>Clon con CH340 sirve</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>El firmware usa los pines extra del Mega (ver firmware/README.md)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -614,7 +622,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Para Arduino Uno</t>
+          <t>Formato UNO, se monta sobre el Mega</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -644,7 +652,11 @@
           <t>Pinza</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>No aplica con el cabezal de disco: se reemplaza por un micro servo SG90 (levante del plumón)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -836,7 +848,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Para eje de 10 mm</t>
+          <t>10 x 19 x 29 mm</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
@@ -850,7 +862,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Rodamiento axial</t>
+          <t>Rodamiento axial 51108</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -863,7 +875,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Primera articulación</t>
+          <t>J1: uno a cada lado de la base</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
@@ -876,11 +888,11 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Rodamiento axial</t>
+          <t>Rodamiento axial 51107</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -889,10 +901,14 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Segunda y tercera articulación</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr"/>
+          <t>J2 y J3: uno arriba y otro abajo de cada brazo</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>La lista del artículo dice 2, pero el ensamble y el STEP usan 4</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -902,7 +918,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Rodamiento radial</t>
+          <t>Rodamiento radial 6807-2RS (61807)</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -910,7 +926,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>35 x 47 mm</t>
+          <t>35 x 47 x 7 mm</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -918,7 +934,11 @@
           <t>Primera articulación</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>No aparece en la lista del artículo; el texto lo monta primero en la base</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -928,7 +948,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Rodamiento radial</t>
+          <t>Rodamiento radial 6806-2RS (61806)</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -936,12 +956,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>30 x 42 mm</t>
+          <t>30 x 42 x 7 mm</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Segunda y tercera articulación</t>
+          <t>J2 y J3: uno dentro de cada brazo</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
@@ -967,7 +987,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Poleas intermedias</t>
+          <t>2 polea intermedia J1, 2 polea intermedia J2, 1 husillo Z</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1266,7 +1286,11 @@
           <t>Guías de pinza</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>No aplica con el cabezal de disco</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1288,7 +1312,11 @@
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>No aplica con el cabezal de disco</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1310,7 +1338,11 @@
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
-      <c r="F37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>No aplica con el cabezal de disco</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">

</xml_diff>